<commit_message>
fix: audit platform figures, report raw vs cleaned MD&A words, and scale percentages
</commit_message>
<xml_diff>
--- a/AAPL_Financial_Analysis.xlsx
+++ b/AAPL_Financial_Analysis.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentiment Analysis" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Price" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Price" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentiment Analysis" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="13"/>
   <chart>
     <title>
       <tx>
@@ -5251,510 +5250,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>AAPL — LOUGHRAN-MCDONALD FINANCIAL SENTIMENT ANALYSIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Item 7 (MD&amp;A) Natural Language Processing — Loughran-McDonald Lexicon (2011)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Fiscal Year</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>Total Words</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>Positive Count</t>
-        </is>
-      </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>Negative Count</t>
-        </is>
-      </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>Net Score</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>P/N Ratio</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Net Sentiment %</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Uncertainty Count</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
-        <is>
-          <t>Litigious Count</t>
-        </is>
-      </c>
-      <c r="J3" s="20" t="inlineStr">
-        <is>
-          <t>Strong Modal</t>
-        </is>
-      </c>
-      <c r="K3" s="20" t="inlineStr">
-        <is>
-          <t>Weak Modal</t>
-        </is>
-      </c>
-      <c r="L3" s="20" t="inlineStr">
-        <is>
-          <t>Tone Classification</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="21" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B4" s="22" t="n">
-        <v>5068</v>
-      </c>
-      <c r="C4" s="22" t="n">
-        <v>132</v>
-      </c>
-      <c r="D4" s="22" t="n">
-        <v>176</v>
-      </c>
-      <c r="E4" s="22" t="n">
-        <v>-44</v>
-      </c>
-      <c r="F4" s="23" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G4" s="24" t="n">
-        <v>-0.008682</v>
-      </c>
-      <c r="H4" s="22" t="n">
-        <v>126</v>
-      </c>
-      <c r="I4" s="22" t="n">
-        <v>53</v>
-      </c>
-      <c r="J4" s="22" t="n">
-        <v>22</v>
-      </c>
-      <c r="K4" s="22" t="n">
-        <v>24</v>
-      </c>
-      <c r="L4" s="25" t="inlineStr">
-        <is>
-          <t>Cautious / Negative</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="26" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B5" s="27" t="n">
-        <v>5234</v>
-      </c>
-      <c r="C5" s="27" t="n">
-        <v>120</v>
-      </c>
-      <c r="D5" s="27" t="n">
-        <v>179</v>
-      </c>
-      <c r="E5" s="27" t="n">
-        <v>-59</v>
-      </c>
-      <c r="F5" s="28" t="n">
-        <v>0.6704</v>
-      </c>
-      <c r="G5" s="29" t="n">
-        <v>-0.011272</v>
-      </c>
-      <c r="H5" s="27" t="n">
-        <v>130</v>
-      </c>
-      <c r="I5" s="27" t="n">
-        <v>50</v>
-      </c>
-      <c r="J5" s="27" t="n">
-        <v>29</v>
-      </c>
-      <c r="K5" s="27" t="n">
-        <v>29</v>
-      </c>
-      <c r="L5" s="25" t="inlineStr">
-        <is>
-          <t>Cautious / Negative</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="21" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B6" s="22" t="n">
-        <v>5031</v>
-      </c>
-      <c r="C6" s="22" t="n">
-        <v>127</v>
-      </c>
-      <c r="D6" s="22" t="n">
-        <v>142</v>
-      </c>
-      <c r="E6" s="22" t="n">
-        <v>-15</v>
-      </c>
-      <c r="F6" s="23" t="n">
-        <v>0.8944</v>
-      </c>
-      <c r="G6" s="24" t="n">
-        <v>-0.002982</v>
-      </c>
-      <c r="H6" s="22" t="n">
-        <v>120</v>
-      </c>
-      <c r="I6" s="22" t="n">
-        <v>54</v>
-      </c>
-      <c r="J6" s="22" t="n">
-        <v>25</v>
-      </c>
-      <c r="K6" s="22" t="n">
-        <v>32</v>
-      </c>
-      <c r="L6" s="25" t="inlineStr">
-        <is>
-          <t>Cautious / Negative</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="26" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B7" s="27" t="n">
-        <v>2962</v>
-      </c>
-      <c r="C7" s="27" t="n">
-        <v>57</v>
-      </c>
-      <c r="D7" s="27" t="n">
-        <v>92</v>
-      </c>
-      <c r="E7" s="27" t="n">
-        <v>-35</v>
-      </c>
-      <c r="F7" s="28" t="n">
-        <v>0.6196</v>
-      </c>
-      <c r="G7" s="29" t="n">
-        <v>-0.011816</v>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>64</v>
-      </c>
-      <c r="I7" s="27" t="n">
-        <v>32</v>
-      </c>
-      <c r="J7" s="27" t="n">
-        <v>10</v>
-      </c>
-      <c r="K7" s="27" t="n">
-        <v>14</v>
-      </c>
-      <c r="L7" s="25" t="inlineStr">
-        <is>
-          <t>Cautious / Negative</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="21" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B8" s="22" t="n">
-        <v>2784</v>
-      </c>
-      <c r="C8" s="22" t="n">
-        <v>51</v>
-      </c>
-      <c r="D8" s="22" t="n">
-        <v>96</v>
-      </c>
-      <c r="E8" s="22" t="n">
-        <v>-45</v>
-      </c>
-      <c r="F8" s="23" t="n">
-        <v>0.5312</v>
-      </c>
-      <c r="G8" s="24" t="n">
-        <v>-0.016164</v>
-      </c>
-      <c r="H8" s="22" t="n">
-        <v>61</v>
-      </c>
-      <c r="I8" s="22" t="n">
-        <v>26</v>
-      </c>
-      <c r="J8" s="22" t="n">
-        <v>10</v>
-      </c>
-      <c r="K8" s="22" t="n">
-        <v>13</v>
-      </c>
-      <c r="L8" s="25" t="inlineStr">
-        <is>
-          <t>Cautious / Negative</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="26" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B9" s="27" t="n">
-        <v>1626</v>
-      </c>
-      <c r="C9" s="27" t="n">
-        <v>49</v>
-      </c>
-      <c r="D9" s="27" t="n">
-        <v>31</v>
-      </c>
-      <c r="E9" s="27" t="n">
-        <v>18</v>
-      </c>
-      <c r="F9" s="28" t="n">
-        <v>1.5806</v>
-      </c>
-      <c r="G9" s="29" t="n">
-        <v>0.01107</v>
-      </c>
-      <c r="H9" s="27" t="n">
-        <v>32</v>
-      </c>
-      <c r="I9" s="27" t="n">
-        <v>14</v>
-      </c>
-      <c r="J9" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="K9" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" s="30" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="21" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B10" s="22" t="n">
-        <v>1542</v>
-      </c>
-      <c r="C10" s="22" t="n">
-        <v>39</v>
-      </c>
-      <c r="D10" s="22" t="n">
-        <v>43</v>
-      </c>
-      <c r="E10" s="22" t="n">
-        <v>-4</v>
-      </c>
-      <c r="F10" s="23" t="n">
-        <v>0.907</v>
-      </c>
-      <c r="G10" s="24" t="n">
-        <v>-0.002594</v>
-      </c>
-      <c r="H10" s="22" t="n">
-        <v>24</v>
-      </c>
-      <c r="I10" s="22" t="n">
-        <v>13</v>
-      </c>
-      <c r="J10" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" s="25" t="inlineStr">
-        <is>
-          <t>Cautious / Negative</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="26" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B11" s="27" t="n">
-        <v>1358</v>
-      </c>
-      <c r="C11" s="27" t="n">
-        <v>24</v>
-      </c>
-      <c r="D11" s="27" t="n">
-        <v>46</v>
-      </c>
-      <c r="E11" s="27" t="n">
-        <v>-22</v>
-      </c>
-      <c r="F11" s="28" t="n">
-        <v>0.5217000000000001</v>
-      </c>
-      <c r="G11" s="29" t="n">
-        <v>-0.0162</v>
-      </c>
-      <c r="H11" s="27" t="n">
-        <v>23</v>
-      </c>
-      <c r="I11" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="J11" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="K11" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="L11" s="25" t="inlineStr">
-        <is>
-          <t>Cautious / Negative</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="21" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B12" s="22" t="n">
-        <v>1338</v>
-      </c>
-      <c r="C12" s="22" t="n">
-        <v>26</v>
-      </c>
-      <c r="D12" s="22" t="n">
-        <v>34</v>
-      </c>
-      <c r="E12" s="22" t="n">
-        <v>-8</v>
-      </c>
-      <c r="F12" s="23" t="n">
-        <v>0.7647</v>
-      </c>
-      <c r="G12" s="24" t="n">
-        <v>-0.005979</v>
-      </c>
-      <c r="H12" s="22" t="n">
-        <v>23</v>
-      </c>
-      <c r="I12" s="22" t="n">
-        <v>13</v>
-      </c>
-      <c r="J12" s="22" t="n">
-        <v>9</v>
-      </c>
-      <c r="K12" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="L12" s="25" t="inlineStr">
-        <is>
-          <t>Cautious / Negative</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="26" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B13" s="27" t="n">
-        <v>1569</v>
-      </c>
-      <c r="C13" s="27" t="n">
-        <v>32</v>
-      </c>
-      <c r="D13" s="27" t="n">
-        <v>37</v>
-      </c>
-      <c r="E13" s="27" t="n">
-        <v>-5</v>
-      </c>
-      <c r="F13" s="28" t="n">
-        <v>0.8649</v>
-      </c>
-      <c r="G13" s="29" t="n">
-        <v>-0.003187</v>
-      </c>
-      <c r="H13" s="27" t="n">
-        <v>29</v>
-      </c>
-      <c r="I13" s="27" t="n">
-        <v>13</v>
-      </c>
-      <c r="J13" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="K13" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="L13" s="25" t="inlineStr">
-        <is>
-          <t>Cautious / Negative</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6123,4 +5618,544 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AAPL — LOUGHRAN-MCDONALD FINANCIAL SENTIMENT ANALYSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Item 7 (MD&amp;A) Natural Language Processing — Loughran-McDonald Lexicon (2011)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Fiscal Year</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>Raw MD&amp;A Words</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>Cleaned MD&amp;A Words</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>Positive Count</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>Negative Count</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>Net Score</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>P/N Ratio</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>Net Sentiment %</t>
+        </is>
+      </c>
+      <c r="I3" s="20" t="inlineStr">
+        <is>
+          <t>Uncertainty Count</t>
+        </is>
+      </c>
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>Litigious Count</t>
+        </is>
+      </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>Strong Modal</t>
+        </is>
+      </c>
+      <c r="L3" s="20" t="inlineStr">
+        <is>
+          <t>Weak Modal</t>
+        </is>
+      </c>
+      <c r="M3" s="20" t="inlineStr">
+        <is>
+          <t>Tone Classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="21" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B4" s="22" t="n">
+        <v>9194</v>
+      </c>
+      <c r="C4" s="22" t="n">
+        <v>5068</v>
+      </c>
+      <c r="D4" s="22" t="n">
+        <v>132</v>
+      </c>
+      <c r="E4" s="22" t="n">
+        <v>176</v>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>-44</v>
+      </c>
+      <c r="G4" s="23" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H4" s="24" t="n">
+        <v>-0.008699999999999999</v>
+      </c>
+      <c r="I4" s="22" t="n">
+        <v>126</v>
+      </c>
+      <c r="J4" s="22" t="n">
+        <v>53</v>
+      </c>
+      <c r="K4" s="22" t="n">
+        <v>22</v>
+      </c>
+      <c r="L4" s="22" t="n">
+        <v>24</v>
+      </c>
+      <c r="M4" s="25" t="inlineStr">
+        <is>
+          <t>Cautious / Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="26" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B5" s="27" t="n">
+        <v>9411</v>
+      </c>
+      <c r="C5" s="27" t="n">
+        <v>5234</v>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>120</v>
+      </c>
+      <c r="E5" s="27" t="n">
+        <v>179</v>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>-59</v>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>0.6704</v>
+      </c>
+      <c r="H5" s="29" t="n">
+        <v>-0.0113</v>
+      </c>
+      <c r="I5" s="27" t="n">
+        <v>130</v>
+      </c>
+      <c r="J5" s="27" t="n">
+        <v>50</v>
+      </c>
+      <c r="K5" s="27" t="n">
+        <v>29</v>
+      </c>
+      <c r="L5" s="27" t="n">
+        <v>29</v>
+      </c>
+      <c r="M5" s="25" t="inlineStr">
+        <is>
+          <t>Cautious / Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="21" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B6" s="22" t="n">
+        <v>8955</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>5031</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>127</v>
+      </c>
+      <c r="E6" s="22" t="n">
+        <v>142</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>-15</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>0.8944</v>
+      </c>
+      <c r="H6" s="24" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="I6" s="22" t="n">
+        <v>120</v>
+      </c>
+      <c r="J6" s="22" t="n">
+        <v>54</v>
+      </c>
+      <c r="K6" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="L6" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="M6" s="25" t="inlineStr">
+        <is>
+          <t>Cautious / Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="26" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>5249</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>2962</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>57</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>92</v>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>-35</v>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>0.6196</v>
+      </c>
+      <c r="H7" s="29" t="n">
+        <v>-0.0118</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>64</v>
+      </c>
+      <c r="J7" s="27" t="n">
+        <v>32</v>
+      </c>
+      <c r="K7" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="L7" s="27" t="n">
+        <v>14</v>
+      </c>
+      <c r="M7" s="25" t="inlineStr">
+        <is>
+          <t>Cautious / Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="21" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>4923</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>2784</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>51</v>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>96</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>-45</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>0.5312</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <v>-0.0162</v>
+      </c>
+      <c r="I8" s="22" t="n">
+        <v>61</v>
+      </c>
+      <c r="J8" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="K8" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="M8" s="25" t="inlineStr">
+        <is>
+          <t>Cautious / Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="26" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B9" s="27" t="n">
+        <v>2925</v>
+      </c>
+      <c r="C9" s="27" t="n">
+        <v>1626</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>31</v>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>1.5806</v>
+      </c>
+      <c r="H9" s="29" t="n">
+        <v>0.0111</v>
+      </c>
+      <c r="I9" s="27" t="n">
+        <v>32</v>
+      </c>
+      <c r="J9" s="27" t="n">
+        <v>14</v>
+      </c>
+      <c r="K9" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="30" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="21" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B10" s="22" t="n">
+        <v>2768</v>
+      </c>
+      <c r="C10" s="22" t="n">
+        <v>1542</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="E10" s="22" t="n">
+        <v>43</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>-4</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <v>-0.0026</v>
+      </c>
+      <c r="I10" s="22" t="n">
+        <v>24</v>
+      </c>
+      <c r="J10" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="K10" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="25" t="inlineStr">
+        <is>
+          <t>Cautious / Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="26" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B11" s="27" t="n">
+        <v>2487</v>
+      </c>
+      <c r="C11" s="27" t="n">
+        <v>1358</v>
+      </c>
+      <c r="D11" s="27" t="n">
+        <v>24</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <v>46</v>
+      </c>
+      <c r="F11" s="27" t="n">
+        <v>-22</v>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>0.5217000000000001</v>
+      </c>
+      <c r="H11" s="29" t="n">
+        <v>-0.0162</v>
+      </c>
+      <c r="I11" s="27" t="n">
+        <v>23</v>
+      </c>
+      <c r="J11" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="K11" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="25" t="inlineStr">
+        <is>
+          <t>Cautious / Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="21" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B12" s="22" t="n">
+        <v>2441</v>
+      </c>
+      <c r="C12" s="22" t="n">
+        <v>1338</v>
+      </c>
+      <c r="D12" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="E12" s="22" t="n">
+        <v>34</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <v>-8</v>
+      </c>
+      <c r="G12" s="23" t="n">
+        <v>0.7647</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="I12" s="22" t="n">
+        <v>23</v>
+      </c>
+      <c r="J12" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="K12" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="L12" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" s="25" t="inlineStr">
+        <is>
+          <t>Cautious / Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="26" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B13" s="27" t="n">
+        <v>2805</v>
+      </c>
+      <c r="C13" s="27" t="n">
+        <v>1569</v>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>32</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <v>37</v>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>-5</v>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>0.8649</v>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>-0.0032</v>
+      </c>
+      <c r="I13" s="27" t="n">
+        <v>29</v>
+      </c>
+      <c r="J13" s="27" t="n">
+        <v>13</v>
+      </c>
+      <c r="K13" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="L13" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="M13" s="25" t="inlineStr">
+        <is>
+          <t>Cautious / Negative</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>